<commit_message>
chore: refresh final 99 gate evidence
</commit_message>
<xml_diff>
--- a/evaluation/final-99-gate/orchestration-download/files/세이프건설-risk-assessment.xlsx
+++ b/evaluation/final-99-gate/orchestration-download/files/세이프건설-risk-assessment.xlsx
@@ -298,13 +298,13 @@
     <t>- 폭염·고온 신호</t>
   </si>
   <si>
-    <t>여름철 체감온도 연결 보류</t>
+    <t>영향예보 보건(일반인) 주의 (울진군평지)</t>
   </si>
   <si>
     <t>- 자외선 신호</t>
   </si>
   <si>
-    <t>자외선지수 1 (낮음) / 실시간 홍반자외선 연결 보류</t>
+    <t>자외선지수 0 (낮음) / 실시간 홍반자외선 연결 보류</t>
   </si>
   <si>
     <t>고온 노출, 직사광선, 탈수, 열탈진·열사병, 자외선 노출, 신규·고령·민감군 작업자 상태 악화</t>

</xml_diff>